<commit_message>
v3.5 expanded course catalog with items in course data table
</commit_message>
<xml_diff>
--- a/course-starter.xlsx
+++ b/course-starter.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\nbs\ag\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A5AA57D-0A54-42A0-9A4B-E11D8B67FAEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B52ABA8-327D-474D-AC14-FAE51D097314}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3720" yWindow="3720" windowWidth="19200" windowHeight="11440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="58">
   <si>
     <t>Hole</t>
   </si>
@@ -63,67 +63,145 @@
     <t>Always</t>
   </si>
   <si>
-    <t>A long Par 5 with a massive fairway bunker.</t>
-  </si>
-  <si>
     <t>Zone</t>
   </si>
   <si>
-    <t>Layup</t>
-  </si>
-  <si>
     <t>Approach</t>
   </si>
   <si>
-    <t>Safe Layup Zone</t>
-  </si>
-  <si>
     <t>Hazard</t>
   </si>
   <si>
     <t>Bunker</t>
   </si>
   <si>
-    <t>W: 30, D: 20</t>
-  </si>
-  <si>
-    <t>The Great Sand Trap</t>
-  </si>
-  <si>
     <t>Advice</t>
   </si>
   <si>
-    <t>Level 1</t>
-  </si>
-  <si>
     <t>Tee</t>
   </si>
   <si>
-    <t>A long Par 5. Hit it straight and far.</t>
-  </si>
-  <si>
-    <t>Level 2</t>
-  </si>
-  <si>
-    <t>Watch out for the massive bunker at 270 yards covering the center-right.</t>
-  </si>
-  <si>
     <t>Level 3</t>
   </si>
   <si>
-    <t>There is a narrow 15-yard gap to the left of the 270-yard bunker. Aim 10 degrees left to thread the needle and set up an Eagle approach.</t>
-  </si>
-  <si>
-    <t>Trouble_Left</t>
-  </si>
-  <si>
-    <t>You are in the rough, but you have a clear angle past the bunker. If you have the distance, you can go straight for the green.</t>
-  </si>
-  <si>
     <t>Greenside</t>
   </si>
   <si>
-    <t>The green is fast and slopes away from you. Play the ball back in your stance to maximize backspin.</t>
+    <t>A 420-yard par 4. Water runs down the entire left side, while an Oak and Maple tree pinch the landing zone on the right.</t>
+  </si>
+  <si>
+    <t>Safe Drive</t>
+  </si>
+  <si>
+    <t>Water</t>
+  </si>
+  <si>
+    <t>W: 40, D: 250</t>
+  </si>
+  <si>
+    <t>Tree</t>
+  </si>
+  <si>
+    <t>Oak Tree</t>
+  </si>
+  <si>
+    <t>R: 5, H: 25</t>
+  </si>
+  <si>
+    <t>Aim about 5 degrees right to take the water out of play. A slight fade works perfectly here.</t>
+  </si>
+  <si>
+    <t>A 165-yard par 3. The pin is tucked safely on the left, but a bunker fiercely guards the front-right of the green.</t>
+  </si>
+  <si>
+    <t>W: 10, D: 15</t>
+  </si>
+  <si>
+    <t>The pin is tucked front-left. If you aim straight at the flag, the front-right bunker is mostly out of play. Do not miss short.</t>
+  </si>
+  <si>
+    <t>A massive 540-yard par 5. A 40-yard wide bunker sits dead center at 270 yards.</t>
+  </si>
+  <si>
+    <t>W: 40, D: 20</t>
+  </si>
+  <si>
+    <t>There is a narrow 15-yard gap to the left of the 270-yard bunker. Aim about 10 degrees left to thread the needle.</t>
+  </si>
+  <si>
+    <t>The green is fast and slopes away. Play the ball back in your stance to maximize your backspin.</t>
+  </si>
+  <si>
+    <t>A 330-yard driveable par 4. A massive, deep bunker protects the front of the green.</t>
+  </si>
+  <si>
+    <t>W: 30, D: 30</t>
+  </si>
+  <si>
+    <t>Left Woods</t>
+  </si>
+  <si>
+    <t>R: 10, H: 30</t>
+  </si>
+  <si>
+    <t>To hit the elbow of the fairway perfectly, you need about 240 yards of carry aimed straight ahead.</t>
+  </si>
+  <si>
+    <t>A 440-yard dogleg right. A 50-foot tall forest completely blocks the direct line to the green.</t>
+  </si>
+  <si>
+    <t>The Corner Forest</t>
+  </si>
+  <si>
+    <t>R: 15, H: 50</t>
+  </si>
+  <si>
+    <t>Aim left of center about 250 yards out. That gives you a clear angle to the back-right pin. Anything right is dead.</t>
+  </si>
+  <si>
+    <t>A reachable 510-yard par 5. The green is an island peninsula.</t>
+  </si>
+  <si>
+    <t>W: 100, D: 15</t>
+  </si>
+  <si>
+    <t>You have a wide-open fairway for your first two shots. Focus on distance.</t>
+  </si>
+  <si>
+    <t>If the wind is in your face, club up. If you are not confident, aim for the left edge of the green.</t>
+  </si>
+  <si>
+    <t>A brutal 215-yard par 3. A 40-foot tall Guardian Oak stands just short and right of the green.</t>
+  </si>
+  <si>
+    <t>The Guardian Oak</t>
+  </si>
+  <si>
+    <t>R: 8, H: 40</t>
+  </si>
+  <si>
+    <t>W: 15, D: 25</t>
+  </si>
+  <si>
+    <t>The Guardian Oak blocks a direct shot to the right pin. You have to play a high fade around it.</t>
+  </si>
+  <si>
+    <t>A claustrophobic 400-yard par 4. The fairway is only 20 yards wide.</t>
+  </si>
+  <si>
+    <t>R: 12, H: 40</t>
+  </si>
+  <si>
+    <t>Leave the driver in the bag. Hit a 3-Wood or long iron to the 200-yard mark.</t>
+  </si>
+  <si>
+    <t>A terrifying 460-yard finishing hole. A massive lake runs the entire right side.</t>
+  </si>
+  <si>
+    <t>W: 40, D: 380</t>
+  </si>
+  <si>
+    <t>Aim 10 degrees left off the tee to take the lake completely out of play.</t>
   </si>
 </sst>
 </file>
@@ -475,7 +553,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:8" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -504,9 +582,9 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="84.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:8" ht="210.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>8</v>
@@ -519,161 +597,729 @@
       </c>
       <c r="E2" s="2"/>
       <c r="F2" s="2">
-        <v>540</v>
+        <v>420</v>
       </c>
       <c r="G2" s="2"/>
       <c r="H2" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="2">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="2">
-        <v>3</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="C3" s="2" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E3" s="2">
         <v>0</v>
       </c>
       <c r="F3" s="2">
-        <v>440</v>
+        <v>250</v>
       </c>
       <c r="G3" s="2"/>
       <c r="H3" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="2">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="2">
+        <v>-45</v>
+      </c>
+      <c r="F4" s="2">
+        <v>100</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" s="2"/>
+    </row>
+    <row r="5" spans="1:8" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="2">
+        <v>1</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" s="2">
         <v>15</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="2">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="s">
+      <c r="F5" s="2">
+        <v>200</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="182.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="2">
+        <v>1</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>16</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" s="2">
-        <v>10</v>
-      </c>
-      <c r="F4" s="2">
-        <v>270</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="2">
-        <v>3</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="154.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="2">
-        <v>3</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>22</v>
       </c>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
       <c r="H6" s="2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="266.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="210.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
+      <c r="F7" s="2">
+        <v>165</v>
+      </c>
       <c r="G7" s="2"/>
       <c r="H7" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="238.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:8" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="D8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E8" s="2">
+        <v>15</v>
+      </c>
+      <c r="F8" s="2">
+        <v>152</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2" t="s">
-        <v>29</v>
-      </c>
+      <c r="H8" s="2"/>
     </row>
     <row r="9" spans="1:8" ht="224.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="E9" s="2"/>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
       <c r="H9" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="154.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="2">
+        <v>3</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2">
+        <v>540</v>
+      </c>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="2">
+        <v>3</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E11" s="2">
+        <v>0</v>
+      </c>
+      <c r="F11" s="2">
+        <v>270</v>
+      </c>
+      <c r="G11" s="2" t="s">
         <v>31</v>
+      </c>
+      <c r="H11" s="2"/>
+    </row>
+    <row r="12" spans="1:8" ht="210.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="2">
+        <v>3</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="196.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="2">
+        <v>3</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="154.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="2">
+        <v>4</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2">
+        <v>330</v>
+      </c>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A15" s="2">
+        <v>4</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E15" s="2">
+        <v>0</v>
+      </c>
+      <c r="F15" s="2">
+        <v>290</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H15" s="2"/>
+    </row>
+    <row r="16" spans="1:8" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="2">
+        <v>4</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E16" s="2">
+        <v>-15</v>
+      </c>
+      <c r="F16" s="2">
+        <v>250</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="210.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A17" s="2">
+        <v>4</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E17" s="2"/>
+      <c r="F17" s="2"/>
+      <c r="G17" s="2"/>
+      <c r="H17" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="210.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A18" s="2">
+        <v>5</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2">
+        <v>440</v>
+      </c>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A19" s="2">
+        <v>5</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E19" s="2">
+        <v>20</v>
+      </c>
+      <c r="F19" s="2">
+        <v>260</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="210.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A20" s="2">
+        <v>5</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E20" s="2"/>
+      <c r="F20" s="2"/>
+      <c r="G20" s="2"/>
+      <c r="H20" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A21" s="2">
+        <v>6</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E21" s="2"/>
+      <c r="F21" s="2">
+        <v>510</v>
+      </c>
+      <c r="G21" s="2"/>
+      <c r="H21" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A22" s="2">
+        <v>6</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E22" s="2">
+        <v>0</v>
+      </c>
+      <c r="F22" s="2">
+        <v>480</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="H22" s="2"/>
+    </row>
+    <row r="23" spans="1:8" ht="154.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A23" s="2">
+        <v>6</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E23" s="2"/>
+      <c r="F23" s="2"/>
+      <c r="G23" s="2"/>
+      <c r="H23" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="182.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A24" s="2">
+        <v>6</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E24" s="2"/>
+      <c r="F24" s="2"/>
+      <c r="G24" s="2"/>
+      <c r="H24" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="168.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A25" s="2">
+        <v>7</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E25" s="2"/>
+      <c r="F25" s="2">
+        <v>215</v>
+      </c>
+      <c r="G25" s="2"/>
+      <c r="H25" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A26" s="2">
+        <v>7</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E26" s="2">
+        <v>10</v>
+      </c>
+      <c r="F26" s="2">
+        <v>180</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A27" s="2">
+        <v>7</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E27" s="2">
+        <v>-15</v>
+      </c>
+      <c r="F27" s="2">
+        <v>195</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="H27" s="2"/>
+    </row>
+    <row r="28" spans="1:8" ht="196.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A28" s="2">
+        <v>7</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E28" s="2"/>
+      <c r="F28" s="2"/>
+      <c r="G28" s="2"/>
+      <c r="H28" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="140.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A29" s="2">
+        <v>8</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E29" s="2"/>
+      <c r="F29" s="2">
+        <v>400</v>
+      </c>
+      <c r="G29" s="2"/>
+      <c r="H29" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A30" s="2">
+        <v>8</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E30" s="2">
+        <v>-20</v>
+      </c>
+      <c r="F30" s="2">
+        <v>250</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="140.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A31" s="2">
+        <v>8</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E31" s="2"/>
+      <c r="F31" s="2"/>
+      <c r="G31" s="2"/>
+      <c r="H31" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" ht="154.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A32" s="2">
+        <v>9</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E32" s="2"/>
+      <c r="F32" s="2">
+        <v>460</v>
+      </c>
+      <c r="G32" s="2"/>
+      <c r="H32" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A33" s="2">
+        <v>9</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E33" s="2">
+        <v>35</v>
+      </c>
+      <c r="F33" s="2">
+        <v>100</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="H33" s="2"/>
+    </row>
+    <row r="34" spans="1:8" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A34" s="2">
+        <v>9</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E34" s="2"/>
+      <c r="F34" s="2"/>
+      <c r="G34" s="2"/>
+      <c r="H34" s="2" t="s">
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>